<commit_message>
Add Home button to Portfolio Dashboard
</commit_message>
<xml_diff>
--- a/data/Internal_Investments_Dashboard.xlsx
+++ b/data/Internal_Investments_Dashboard.xlsx
@@ -8,12 +8,12 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/mornay/Documents/market-dashboard/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F174F1B3-D78C-C947-BD89-C7A72954B105}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CABCDABF-B657-854F-A253-B4EEC147B11E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3480" yWindow="2660" windowWidth="27640" windowHeight="16680" xr2:uid="{4930D9E8-EC32-2740-B70C-4A799C618033}"/>
+    <workbookView xWindow="3440" yWindow="2640" windowWidth="27640" windowHeight="16680" xr2:uid="{4930D9E8-EC32-2740-B70C-4A799C618033}"/>
   </bookViews>
   <sheets>
-    <sheet name="Investments Map Data" sheetId="1" r:id="rId1"/>
+    <sheet name="Master Sheet" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="181029"/>
   <extLst>

</xml_diff>

<commit_message>
Updated Grovepoint Invested Status
</commit_message>
<xml_diff>
--- a/data/Internal_Investments_Dashboard.xlsx
+++ b/data/Internal_Investments_Dashboard.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/mornay/Documents/market-dashboard/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CABCDABF-B657-854F-A253-B4EEC147B11E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E584B2A1-CC88-8548-81F2-D1838F096C35}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="3440" yWindow="2640" windowWidth="27640" windowHeight="16680" xr2:uid="{4930D9E8-EC32-2740-B70C-4A799C618033}"/>
   </bookViews>
@@ -1302,7 +1302,7 @@
       <c r="N14" s="14"/>
       <c r="O14" s="14"/>
       <c r="P14" s="16" t="s">
-        <v>44</v>
+        <v>15</v>
       </c>
     </row>
     <row r="15" spans="1:16" ht="35" customHeight="1" x14ac:dyDescent="0.2">

</xml_diff>